<commit_message>
feat: adjusted tables + sorting indicators
</commit_message>
<xml_diff>
--- a/Reference_Table.xlsx
+++ b/Reference_Table.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/edoardociato/TennisAnalyticsV3/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/edoardociato/02_Work/TennisAnalytics_Master/TennisAnalyticsV3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEAD77A7-366C-B846-9198-DBACADD4C889}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90217129-F1CD-474C-9702-1144EDEF8BA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4300" yWindow="780" windowWidth="29900" windowHeight="21460" xr2:uid="{589F79FF-B3DF-4A72-A764-0CD71D5A19DC}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="146">
   <si>
     <t>Description</t>
   </si>
@@ -116,367 +116,364 @@
     <t>2nd_T_Avg</t>
   </si>
   <si>
+    <t>2nd_Wide_Avg</t>
+  </si>
+  <si>
+    <t>Break Pts Saved</t>
+  </si>
+  <si>
+    <t>BP_Saved</t>
+  </si>
+  <si>
+    <t>Break Pts Faced  Games %</t>
+  </si>
+  <si>
+    <t>BPF_Games</t>
+  </si>
+  <si>
+    <t>Games won with Break Pts Faced</t>
+  </si>
+  <si>
+    <t>Hold/BPFG</t>
+  </si>
+  <si>
+    <t>Deuce Aces %</t>
+  </si>
+  <si>
+    <t>Deuce_A%</t>
+  </si>
+  <si>
+    <t>Ad Aces %</t>
+  </si>
+  <si>
+    <t>Ad_A%</t>
+  </si>
+  <si>
+    <t>Deuce Service Pts won %</t>
+  </si>
+  <si>
+    <t>Deuce_SPW%</t>
+  </si>
+  <si>
+    <t>Ad Service Pts won %</t>
+  </si>
+  <si>
+    <t>Ad_SPW%</t>
+  </si>
+  <si>
+    <t>Serve &amp; Volley won%</t>
+  </si>
+  <si>
+    <t>SnV_W%</t>
+  </si>
+  <si>
+    <t>Tactics</t>
+  </si>
+  <si>
+    <t>Service Impact</t>
+  </si>
+  <si>
+    <t>SvImpact</t>
+  </si>
+  <si>
+    <t>Serve Impact 1st</t>
+  </si>
+  <si>
+    <t>SvImpact.1</t>
+  </si>
+  <si>
+    <t>Break %</t>
+  </si>
+  <si>
+    <t>Brk%</t>
+  </si>
+  <si>
+    <t>Return</t>
+  </si>
+  <si>
+    <t>Return Points won</t>
+  </si>
+  <si>
+    <t>RPW</t>
+  </si>
+  <si>
+    <t>Return in Play won %</t>
+  </si>
+  <si>
+    <t>RiP_W%</t>
+  </si>
+  <si>
+    <t>Break Pts converted</t>
+  </si>
+  <si>
+    <t>BP_Conv</t>
+  </si>
+  <si>
+    <t>Break vs Games with Break Pts</t>
+  </si>
+  <si>
+    <t>BP_Conv/BPG</t>
+  </si>
+  <si>
+    <t>Games with Break Pts</t>
+  </si>
+  <si>
+    <t>BP_Games</t>
+  </si>
+  <si>
+    <t>Break Back%</t>
+  </si>
+  <si>
+    <t>BreakBack%</t>
+  </si>
+  <si>
+    <t>Attitude</t>
+  </si>
+  <si>
+    <t>Deuce Return Pts won%</t>
+  </si>
+  <si>
+    <t>Deuce_RPW%</t>
+  </si>
+  <si>
+    <t>Ad Return Pts won %</t>
+  </si>
+  <si>
+    <t>Ad_RPW%</t>
+  </si>
+  <si>
+    <t>Forehand Wnr Pts</t>
+  </si>
+  <si>
+    <t>FH_Wnr/Pt</t>
+  </si>
+  <si>
+    <t>Rally</t>
+  </si>
+  <si>
+    <t>Backhand Wnr Pts</t>
+  </si>
+  <si>
+    <t>BH_Wnr/Pt</t>
+  </si>
+  <si>
+    <t>Winners</t>
+  </si>
+  <si>
+    <t>Wnr/Pt</t>
+  </si>
+  <si>
+    <t>Unforced Errors</t>
+  </si>
+  <si>
+    <t>UFE/Pt</t>
+  </si>
+  <si>
+    <t>Inside Out Winners</t>
+  </si>
+  <si>
+    <t>IO_Wnr%</t>
+  </si>
+  <si>
+    <t>DTL_Wnr%</t>
+  </si>
+  <si>
+    <t>DTL_Wnr%.1</t>
+  </si>
+  <si>
+    <t>Ratio Winners / Unforced</t>
+  </si>
+  <si>
+    <t>Ratio</t>
+  </si>
+  <si>
+    <t>Efficiency</t>
+  </si>
+  <si>
+    <t>Drop:_Freq</t>
+  </si>
+  <si>
+    <t>Net Frequency</t>
+  </si>
+  <si>
+    <t>Net_Freq</t>
+  </si>
+  <si>
+    <t>Serve &amp; Volley  Frequency</t>
+  </si>
+  <si>
+    <t>SnV_Freq</t>
+  </si>
+  <si>
+    <t>ReturnAgg</t>
+  </si>
+  <si>
+    <t>Rally Aggressive</t>
+  </si>
+  <si>
+    <t>RallyAgg</t>
+  </si>
+  <si>
+    <t>Serve StayMatch won</t>
+  </si>
+  <si>
+    <t>SvStayMatch</t>
+  </si>
+  <si>
+    <t>Serve ForMatch won</t>
+  </si>
+  <si>
+    <t>SvForMatch</t>
+  </si>
+  <si>
+    <t>Consol%</t>
+  </si>
+  <si>
+    <t>Tie Break won</t>
+  </si>
+  <si>
+    <t>TB%</t>
+  </si>
+  <si>
+    <t>Dominance Ratio</t>
+  </si>
+  <si>
+    <t>DR</t>
+  </si>
+  <si>
+    <t>Return shallow %</t>
+  </si>
+  <si>
+    <t>shallow</t>
+  </si>
+  <si>
+    <t>Return deep %</t>
+  </si>
+  <si>
+    <t>deep</t>
+  </si>
+  <si>
+    <t>Return very deep %</t>
+  </si>
+  <si>
+    <t>very_deep</t>
+  </si>
+  <si>
+    <t>Return unforced %</t>
+  </si>
+  <si>
+    <t>unforced</t>
+  </si>
+  <si>
+    <t>Cross court %</t>
+  </si>
+  <si>
+    <t>crosscourt</t>
+  </si>
+  <si>
+    <t>Down middle %</t>
+  </si>
+  <si>
+    <t>down_middle</t>
+  </si>
+  <si>
+    <t>Down the Line %</t>
+  </si>
+  <si>
+    <t>down_the_line</t>
+  </si>
+  <si>
+    <t>Inside Out %</t>
+  </si>
+  <si>
+    <t>inside_out</t>
+  </si>
+  <si>
+    <t>Inside In%</t>
+  </si>
+  <si>
+    <t>inside_in</t>
+  </si>
+  <si>
+    <t>Chart</t>
+  </si>
+  <si>
+    <t>Table</t>
+  </si>
+  <si>
+    <t>Categories</t>
+  </si>
+  <si>
+    <t>Down the Line Winners</t>
+  </si>
+  <si>
+    <t>Down the Line Winners 1st</t>
+  </si>
+  <si>
+    <t>reference_table</t>
+  </si>
+  <si>
+    <t>group_004</t>
+  </si>
+  <si>
+    <t>group_009</t>
+  </si>
+  <si>
+    <t>group_010</t>
+  </si>
+  <si>
+    <t>group_011</t>
+  </si>
+  <si>
+    <t>group_012</t>
+  </si>
+  <si>
+    <t>group_016</t>
+  </si>
+  <si>
+    <t>group_013</t>
+  </si>
+  <si>
+    <t>group_014</t>
+  </si>
+  <si>
+    <t>group_008</t>
+  </si>
+  <si>
+    <t>filter_date</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>Match</t>
+  </si>
+  <si>
+    <t>Return Aggressive</t>
+  </si>
+  <si>
+    <t>Break Consolidation %</t>
+  </si>
+  <si>
+    <t>mcp_m_stats_returndepth</t>
+  </si>
+  <si>
+    <t>mcp_m_stats_shotdirection</t>
+  </si>
+  <si>
+    <t>JS</t>
+  </si>
+  <si>
+    <t>1st T Speed</t>
+  </si>
+  <si>
+    <t>2nd T Speed</t>
+  </si>
+  <si>
+    <t>Drop Frequency</t>
+  </si>
+  <si>
     <t>2nd Wide Speed</t>
-  </si>
-  <si>
-    <t>2nd_Wide_Avg</t>
-  </si>
-  <si>
-    <t>Break Pts Saved</t>
-  </si>
-  <si>
-    <t>BP_Saved</t>
-  </si>
-  <si>
-    <t>Break Pts Faced  Games %</t>
-  </si>
-  <si>
-    <t>BPF_Games</t>
-  </si>
-  <si>
-    <t>Games won with Break Pts Faced</t>
-  </si>
-  <si>
-    <t>Hold/BPFG</t>
-  </si>
-  <si>
-    <t>Deuce Aces %</t>
-  </si>
-  <si>
-    <t>Deuce_A%</t>
-  </si>
-  <si>
-    <t>Ad Aces %</t>
-  </si>
-  <si>
-    <t>Ad_A%</t>
-  </si>
-  <si>
-    <t>Deuce Service Pts won %</t>
-  </si>
-  <si>
-    <t>Deuce_SPW%</t>
-  </si>
-  <si>
-    <t>Ad Service Pts won %</t>
-  </si>
-  <si>
-    <t>Ad_SPW%</t>
-  </si>
-  <si>
-    <t>Serve &amp; Volley won%</t>
-  </si>
-  <si>
-    <t>SnV_W%</t>
-  </si>
-  <si>
-    <t>Tactics</t>
-  </si>
-  <si>
-    <t>Service Impact</t>
-  </si>
-  <si>
-    <t>SvImpact</t>
-  </si>
-  <si>
-    <t>Serve Impact 1st</t>
-  </si>
-  <si>
-    <t>SvImpact.1</t>
-  </si>
-  <si>
-    <t>Break %</t>
-  </si>
-  <si>
-    <t>Brk%</t>
-  </si>
-  <si>
-    <t>Return</t>
-  </si>
-  <si>
-    <t>Return Points won</t>
-  </si>
-  <si>
-    <t>RPW</t>
-  </si>
-  <si>
-    <t>Return in Play won %</t>
-  </si>
-  <si>
-    <t>RiP_W%</t>
-  </si>
-  <si>
-    <t>Break Pts converted</t>
-  </si>
-  <si>
-    <t>BP_Conv</t>
-  </si>
-  <si>
-    <t>Break vs Games with Break Pts</t>
-  </si>
-  <si>
-    <t>BP_Conv/BPG</t>
-  </si>
-  <si>
-    <t>Games with Break Pts</t>
-  </si>
-  <si>
-    <t>BP_Games</t>
-  </si>
-  <si>
-    <t>Break Back%</t>
-  </si>
-  <si>
-    <t>BreakBack%</t>
-  </si>
-  <si>
-    <t>Attitude</t>
-  </si>
-  <si>
-    <t>Deuce Return Pts won%</t>
-  </si>
-  <si>
-    <t>Deuce_RPW%</t>
-  </si>
-  <si>
-    <t>Ad Return Pts won %</t>
-  </si>
-  <si>
-    <t>Ad_RPW%</t>
-  </si>
-  <si>
-    <t>Forehand Wnr Pts</t>
-  </si>
-  <si>
-    <t>FH_Wnr/Pt</t>
-  </si>
-  <si>
-    <t>Rally</t>
-  </si>
-  <si>
-    <t>Backhand Wnr Pts</t>
-  </si>
-  <si>
-    <t>BH_Wnr/Pt</t>
-  </si>
-  <si>
-    <t>Winners</t>
-  </si>
-  <si>
-    <t>Wnr/Pt</t>
-  </si>
-  <si>
-    <t>Unforced Errors</t>
-  </si>
-  <si>
-    <t>UFE/Pt</t>
-  </si>
-  <si>
-    <t>Inside Out Winners</t>
-  </si>
-  <si>
-    <t>IO_Wnr%</t>
-  </si>
-  <si>
-    <t>DTL_Wnr%</t>
-  </si>
-  <si>
-    <t>DTL_Wnr%.1</t>
-  </si>
-  <si>
-    <t>Ratio Winners / Unforced</t>
-  </si>
-  <si>
-    <t>Ratio</t>
-  </si>
-  <si>
-    <t>Efficiency</t>
-  </si>
-  <si>
-    <t>Drop Freqency</t>
-  </si>
-  <si>
-    <t>Drop:_Freq</t>
-  </si>
-  <si>
-    <t>Net Frequency</t>
-  </si>
-  <si>
-    <t>Net_Freq</t>
-  </si>
-  <si>
-    <t>Serve &amp; Volley  Frequency</t>
-  </si>
-  <si>
-    <t>SnV_Freq</t>
-  </si>
-  <si>
-    <t>ReturnAgg</t>
-  </si>
-  <si>
-    <t>Rally Aggressive</t>
-  </si>
-  <si>
-    <t>RallyAgg</t>
-  </si>
-  <si>
-    <t>Serve StayMatch won</t>
-  </si>
-  <si>
-    <t>SvStayMatch</t>
-  </si>
-  <si>
-    <t>Serve ForMatch won</t>
-  </si>
-  <si>
-    <t>SvForMatch</t>
-  </si>
-  <si>
-    <t>Consol%</t>
-  </si>
-  <si>
-    <t>Tie Break won</t>
-  </si>
-  <si>
-    <t>TB%</t>
-  </si>
-  <si>
-    <t>Dominance Ratio</t>
-  </si>
-  <si>
-    <t>DR</t>
-  </si>
-  <si>
-    <t>Return shallow %</t>
-  </si>
-  <si>
-    <t>shallow</t>
-  </si>
-  <si>
-    <t>Return deep %</t>
-  </si>
-  <si>
-    <t>deep</t>
-  </si>
-  <si>
-    <t>Return very deep %</t>
-  </si>
-  <si>
-    <t>very_deep</t>
-  </si>
-  <si>
-    <t>Return unforced %</t>
-  </si>
-  <si>
-    <t>unforced</t>
-  </si>
-  <si>
-    <t>Cross court %</t>
-  </si>
-  <si>
-    <t>crosscourt</t>
-  </si>
-  <si>
-    <t>Down middle %</t>
-  </si>
-  <si>
-    <t>down_middle</t>
-  </si>
-  <si>
-    <t>Down the Line %</t>
-  </si>
-  <si>
-    <t>down_the_line</t>
-  </si>
-  <si>
-    <t>Inside Out %</t>
-  </si>
-  <si>
-    <t>inside_out</t>
-  </si>
-  <si>
-    <t>Inside In%</t>
-  </si>
-  <si>
-    <t>inside_in</t>
-  </si>
-  <si>
-    <t>Chart</t>
-  </si>
-  <si>
-    <t>Table</t>
-  </si>
-  <si>
-    <t>Categories</t>
-  </si>
-  <si>
-    <t>Y</t>
-  </si>
-  <si>
-    <t>Down the Line Winners</t>
-  </si>
-  <si>
-    <t>Down the Line Winners 1st</t>
-  </si>
-  <si>
-    <t>reference_table</t>
-  </si>
-  <si>
-    <t>group_004</t>
-  </si>
-  <si>
-    <t>group_009</t>
-  </si>
-  <si>
-    <t>group_010</t>
-  </si>
-  <si>
-    <t>group_011</t>
-  </si>
-  <si>
-    <t>group_012</t>
-  </si>
-  <si>
-    <t>group_016</t>
-  </si>
-  <si>
-    <t>group_013</t>
-  </si>
-  <si>
-    <t>group_014</t>
-  </si>
-  <si>
-    <t>group_008</t>
-  </si>
-  <si>
-    <t>filter_date</t>
-  </si>
-  <si>
-    <t>Year</t>
-  </si>
-  <si>
-    <t>Match</t>
-  </si>
-  <si>
-    <t>Return Aggressive</t>
-  </si>
-  <si>
-    <t>Break Consolidation %</t>
-  </si>
-  <si>
-    <t>mcp_m_stats_returndepth</t>
-  </si>
-  <si>
-    <t>mcp_m_stats_shotdirection</t>
-  </si>
-  <si>
-    <t>JS</t>
-  </si>
-  <si>
-    <t>1st T Speed</t>
-  </si>
-  <si>
-    <t>2nd T Speed</t>
   </si>
 </sst>
 </file>
@@ -716,14 +713,14 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>11</xdr:col>
+      <xdr:col>12</xdr:col>
       <xdr:colOff>243840</xdr:colOff>
       <xdr:row>40</xdr:row>
       <xdr:rowOff>30480</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>284373</xdr:colOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>386286</xdr:colOff>
       <xdr:row>50</xdr:row>
       <xdr:rowOff>164104</xdr:rowOff>
     </xdr:to>
@@ -760,13 +757,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>17</xdr:col>
+      <xdr:col>18</xdr:col>
       <xdr:colOff>326554</xdr:colOff>
       <xdr:row>40</xdr:row>
       <xdr:rowOff>61564</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>23</xdr:col>
+      <xdr:col>24</xdr:col>
       <xdr:colOff>426720</xdr:colOff>
       <xdr:row>66</xdr:row>
       <xdr:rowOff>174126</xdr:rowOff>
@@ -804,14 +801,14 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>11</xdr:col>
+      <xdr:col>12</xdr:col>
       <xdr:colOff>304214</xdr:colOff>
       <xdr:row>53</xdr:row>
       <xdr:rowOff>137160</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>196793</xdr:colOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>298706</xdr:colOff>
       <xdr:row>66</xdr:row>
       <xdr:rowOff>40368</xdr:rowOff>
     </xdr:to>
@@ -848,13 +845,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>23</xdr:col>
+      <xdr:col>24</xdr:col>
       <xdr:colOff>507172</xdr:colOff>
       <xdr:row>41</xdr:row>
       <xdr:rowOff>15240</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>30</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>17699</xdr:colOff>
       <xdr:row>56</xdr:row>
       <xdr:rowOff>80422</xdr:rowOff>
@@ -894,9 +891,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4CF2A204-07DE-4E13-A729-0914269FED17}" name="Table1" displayName="Table1" ref="A2:J61" totalsRowShown="0" headerRowDxfId="2" headerRowBorderDxfId="1" tableBorderDxfId="0">
-  <autoFilter ref="A2:J61" xr:uid="{4CF2A204-07DE-4E13-A729-0914269FED17}"/>
-  <tableColumns count="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4CF2A204-07DE-4E13-A729-0914269FED17}" name="Table1" displayName="Table1" ref="A2:K61" totalsRowShown="0" headerRowDxfId="2" headerRowBorderDxfId="1" tableBorderDxfId="0">
+  <autoFilter ref="A2:K61" xr:uid="{4CF2A204-07DE-4E13-A729-0914269FED17}"/>
+  <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{DCA3A328-43A0-4C5B-8661-6C80084ACF61}" name="variable"/>
     <tableColumn id="4" xr3:uid="{6999234A-287D-4816-9670-BB216BACB7D2}" name="Parity"/>
     <tableColumn id="7" xr3:uid="{5670A2A2-7A52-4F3B-A053-13F1C166238A}" name="Description"/>
@@ -907,6 +904,7 @@
     <tableColumn id="5" xr3:uid="{1456AE88-D6C9-094E-B500-FFA5B431E02F}" name="reference_table"/>
     <tableColumn id="11" xr3:uid="{B8AF6EE2-443C-224D-AE4E-26A832BCCE0C}" name="filter_date"/>
     <tableColumn id="6" xr3:uid="{82526720-49F1-5C4C-98C4-4BA387B0AFB7}" name="JS"/>
+    <tableColumn id="10" xr3:uid="{D7F34036-C7F2-8445-B0C4-36725F114B8C}" name="Ratio"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1229,7 +1227,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C70B48F9-3C73-4604-B662-B76B4FE5C262}">
-  <dimension ref="A2:L61"/>
+  <dimension ref="A2:M61"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.6640625" customWidth="1"/>
@@ -1244,7 +1242,7 @@
     <col min="12" max="12" width="10.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -1258,28 +1256,31 @@
         <v>3</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="G2" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="M2" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="H2" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="L2" s="7" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -1302,16 +1303,22 @@
         <v>1</v>
       </c>
       <c r="H3" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="I3" t="s">
-        <v>138</v>
-      </c>
-      <c r="L3" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>1</v>
+      </c>
+      <c r="M3" s="8" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -1334,16 +1341,22 @@
         <v>1</v>
       </c>
       <c r="H4" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="I4" t="s">
-        <v>138</v>
-      </c>
-      <c r="L4" s="8" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+        <v>135</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>1</v>
+      </c>
+      <c r="M4" s="8" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1366,16 +1379,22 @@
         <v>1</v>
       </c>
       <c r="H5" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="I5" t="s">
-        <v>138</v>
-      </c>
-      <c r="L5" s="8" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+        <v>135</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>1</v>
+      </c>
+      <c r="M5" s="8" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -1398,16 +1417,22 @@
         <v>1</v>
       </c>
       <c r="H6" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="I6" t="s">
-        <v>138</v>
-      </c>
-      <c r="L6" s="8" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+        <v>135</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>1</v>
+      </c>
+      <c r="M6" s="8" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -1430,16 +1455,22 @@
         <v>1</v>
       </c>
       <c r="H7" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="I7" t="s">
-        <v>138</v>
-      </c>
-      <c r="L7" s="8" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+        <v>135</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
+        <v>1</v>
+      </c>
+      <c r="M7" s="8" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -1462,16 +1493,22 @@
         <v>1</v>
       </c>
       <c r="H8" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="I8" t="s">
-        <v>138</v>
-      </c>
-      <c r="L8" s="8" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+        <v>135</v>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8">
+        <v>1</v>
+      </c>
+      <c r="M8" s="8" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>17</v>
       </c>
@@ -1494,13 +1531,19 @@
         <v>1</v>
       </c>
       <c r="H9" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="I9" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+        <v>135</v>
+      </c>
+      <c r="J9">
+        <v>0</v>
+      </c>
+      <c r="K9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -1523,13 +1566,19 @@
         <v>0</v>
       </c>
       <c r="H10" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="I10" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="J10">
+        <v>0</v>
+      </c>
+      <c r="K10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>20</v>
       </c>
@@ -1537,7 +1586,7 @@
         <v>1</v>
       </c>
       <c r="C11" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="D11" t="s">
         <v>5</v>
@@ -1552,13 +1601,19 @@
         <v>0</v>
       </c>
       <c r="H11" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="I11" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
+      <c r="K11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>22</v>
       </c>
@@ -1581,13 +1636,19 @@
         <v>0</v>
       </c>
       <c r="H12" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="I12" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
+      <c r="K12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>24</v>
       </c>
@@ -1610,13 +1671,19 @@
         <v>0</v>
       </c>
       <c r="H13" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="I13" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="J13">
+        <v>0</v>
+      </c>
+      <c r="K13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>25</v>
       </c>
@@ -1624,7 +1691,7 @@
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="D14" t="s">
         <v>5</v>
@@ -1639,21 +1706,27 @@
         <v>0</v>
       </c>
       <c r="H14" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="I14" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="J14">
+        <v>0</v>
+      </c>
+      <c r="K14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B15">
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>26</v>
+        <v>145</v>
       </c>
       <c r="D15" t="s">
         <v>5</v>
@@ -1668,21 +1741,27 @@
         <v>0</v>
       </c>
       <c r="H15" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="I15" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="J15">
+        <v>0</v>
+      </c>
+      <c r="K15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B16">
         <v>1</v>
       </c>
       <c r="C16" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D16" t="s">
         <v>5</v>
@@ -1697,21 +1776,27 @@
         <v>0</v>
       </c>
       <c r="H16" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="I16" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="J16">
+        <v>0</v>
+      </c>
+      <c r="K16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B17">
         <v>-1</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D17" t="s">
         <v>5</v>
@@ -1726,21 +1811,27 @@
         <v>0</v>
       </c>
       <c r="H17" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="I17" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="J17">
+        <v>0</v>
+      </c>
+      <c r="K17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B18">
         <v>1</v>
       </c>
       <c r="C18" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D18" t="s">
         <v>5</v>
@@ -1755,21 +1846,27 @@
         <v>0</v>
       </c>
       <c r="H18" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="I18" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="J18">
+        <v>0</v>
+      </c>
+      <c r="K18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B19">
         <v>1</v>
       </c>
       <c r="C19" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D19" t="s">
         <v>5</v>
@@ -1784,21 +1881,27 @@
         <v>0</v>
       </c>
       <c r="H19" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="I19" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="J19">
+        <v>0</v>
+      </c>
+      <c r="K19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B20">
         <v>1</v>
       </c>
       <c r="C20" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D20" t="s">
         <v>5</v>
@@ -1813,21 +1916,27 @@
         <v>0</v>
       </c>
       <c r="H20" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="I20" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="J20">
+        <v>0</v>
+      </c>
+      <c r="K20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B21">
         <v>1</v>
       </c>
       <c r="C21" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D21" t="s">
         <v>5</v>
@@ -1842,21 +1951,27 @@
         <v>0</v>
       </c>
       <c r="H21" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="I21" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="J21">
+        <v>0</v>
+      </c>
+      <c r="K21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B22">
         <v>1</v>
       </c>
       <c r="C22" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D22" t="s">
         <v>5</v>
@@ -1871,21 +1986,27 @@
         <v>0</v>
       </c>
       <c r="H22" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="I22" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="J22">
+        <v>0</v>
+      </c>
+      <c r="K22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B23">
         <v>1</v>
       </c>
       <c r="C23" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D23" t="s">
         <v>5</v>
@@ -1900,21 +2021,27 @@
         <v>0</v>
       </c>
       <c r="H23" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="I23" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="J23">
+        <v>0</v>
+      </c>
+      <c r="K23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B24">
         <v>1</v>
       </c>
       <c r="C24" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D24" t="s">
         <v>5</v>
@@ -1929,21 +2056,27 @@
         <v>0</v>
       </c>
       <c r="H24" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="I24" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="J24">
+        <v>0</v>
+      </c>
+      <c r="K24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B25">
         <v>1</v>
       </c>
       <c r="C25" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D25" t="s">
         <v>5</v>
@@ -1958,53 +2091,65 @@
         <v>0</v>
       </c>
       <c r="H25" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="I25" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="J25">
+        <v>0</v>
+      </c>
+      <c r="K25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
+        <v>49</v>
+      </c>
+      <c r="B26">
+        <v>1</v>
+      </c>
+      <c r="C26" t="s">
+        <v>48</v>
+      </c>
+      <c r="D26" t="s">
         <v>50</v>
       </c>
-      <c r="B26">
-        <v>1</v>
-      </c>
-      <c r="C26" t="s">
-        <v>49</v>
-      </c>
-      <c r="D26" t="s">
+      <c r="E26">
+        <v>0</v>
+      </c>
+      <c r="F26" s="6">
+        <v>1</v>
+      </c>
+      <c r="G26">
+        <v>1</v>
+      </c>
+      <c r="H26" t="s">
+        <v>125</v>
+      </c>
+      <c r="I26" t="s">
+        <v>135</v>
+      </c>
+      <c r="J26">
+        <v>0</v>
+      </c>
+      <c r="K26">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>52</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="E26">
-        <v>0</v>
-      </c>
-      <c r="F26" s="6">
-        <v>1</v>
-      </c>
-      <c r="G26">
-        <v>1</v>
-      </c>
-      <c r="H26" t="s">
-        <v>128</v>
-      </c>
-      <c r="I26" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A27" t="s">
-        <v>53</v>
-      </c>
-      <c r="B27">
-        <v>1</v>
-      </c>
-      <c r="C27" s="5" t="s">
-        <v>52</v>
-      </c>
       <c r="D27" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E27">
         <v>1</v>
@@ -2016,24 +2161,30 @@
         <v>1</v>
       </c>
       <c r="H27" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="I27" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
+        <v>135</v>
+      </c>
+      <c r="J27">
+        <v>0</v>
+      </c>
+      <c r="K27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B28">
         <v>1</v>
       </c>
       <c r="C28" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D28" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E28">
         <v>0</v>
@@ -2045,24 +2196,30 @@
         <v>1</v>
       </c>
       <c r="H28" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="I28" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="J28">
+        <v>0</v>
+      </c>
+      <c r="K28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B29">
         <v>1</v>
       </c>
       <c r="C29" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D29" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E29">
         <v>0</v>
@@ -2074,24 +2231,30 @@
         <v>1</v>
       </c>
       <c r="H29" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="I29" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="J29">
+        <v>0</v>
+      </c>
+      <c r="K29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B30">
         <v>1</v>
       </c>
       <c r="C30" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D30" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E30">
         <v>1</v>
@@ -2103,24 +2266,30 @@
         <v>1</v>
       </c>
       <c r="H30" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="I30" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="J30">
+        <v>0</v>
+      </c>
+      <c r="K30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B31">
         <v>1</v>
       </c>
       <c r="C31" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D31" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E31">
         <v>1</v>
@@ -2132,24 +2301,30 @@
         <v>1</v>
       </c>
       <c r="H31" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="I31" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="J31">
+        <v>0</v>
+      </c>
+      <c r="K31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
+        <v>62</v>
+      </c>
+      <c r="B32">
+        <v>1</v>
+      </c>
+      <c r="C32" t="s">
+        <v>61</v>
+      </c>
+      <c r="D32" t="s">
         <v>63</v>
-      </c>
-      <c r="B32">
-        <v>1</v>
-      </c>
-      <c r="C32" t="s">
-        <v>62</v>
-      </c>
-      <c r="D32" t="s">
-        <v>64</v>
       </c>
       <c r="E32">
         <v>0</v>
@@ -2161,24 +2336,30 @@
         <v>1</v>
       </c>
       <c r="H32" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="I32" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="J32">
+        <v>0</v>
+      </c>
+      <c r="K32">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B33">
         <v>1</v>
       </c>
       <c r="C33" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D33" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E33">
         <v>0</v>
@@ -2190,24 +2371,30 @@
         <v>1</v>
       </c>
       <c r="H33" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="I33" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="J33">
+        <v>0</v>
+      </c>
+      <c r="K33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B34">
         <v>1</v>
       </c>
       <c r="C34" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D34" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E34">
         <v>0</v>
@@ -2219,24 +2406,30 @@
         <v>1</v>
       </c>
       <c r="H34" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="I34" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="J34">
+        <v>0</v>
+      </c>
+      <c r="K34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
+        <v>69</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>68</v>
+      </c>
+      <c r="D35" t="s">
         <v>70</v>
-      </c>
-      <c r="B35">
-        <v>1</v>
-      </c>
-      <c r="C35" t="s">
-        <v>69</v>
-      </c>
-      <c r="D35" t="s">
-        <v>71</v>
       </c>
       <c r="E35">
         <v>0</v>
@@ -2248,24 +2441,30 @@
         <v>1</v>
       </c>
       <c r="H35" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="I35" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="J35">
+        <v>0</v>
+      </c>
+      <c r="K35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B36">
         <v>1</v>
       </c>
       <c r="C36" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D36" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E36">
         <v>0</v>
@@ -2277,24 +2476,30 @@
         <v>1</v>
       </c>
       <c r="H36" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="I36" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="J36">
+        <v>0</v>
+      </c>
+      <c r="K36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B37">
         <v>1</v>
       </c>
       <c r="C37" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D37" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E37">
         <v>1</v>
@@ -2306,24 +2511,30 @@
         <v>1</v>
       </c>
       <c r="H37" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="I37" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="J37">
+        <v>0</v>
+      </c>
+      <c r="K37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B38">
         <v>-1</v>
       </c>
       <c r="C38" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D38" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E38">
         <v>1</v>
@@ -2335,24 +2546,30 @@
         <v>1</v>
       </c>
       <c r="H38" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="I38" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="J38">
+        <v>0</v>
+      </c>
+      <c r="K38">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B39">
         <v>1</v>
       </c>
       <c r="C39" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D39" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E39">
         <v>0</v>
@@ -2364,24 +2581,30 @@
         <v>1</v>
       </c>
       <c r="H39" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="I39" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="J39">
+        <v>0</v>
+      </c>
+      <c r="K39">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B40">
         <v>1</v>
       </c>
       <c r="C40" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="D40" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E40">
         <v>0</v>
@@ -2393,24 +2616,30 @@
         <v>1</v>
       </c>
       <c r="H40" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="I40" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="J40">
+        <v>0</v>
+      </c>
+      <c r="K40">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B41">
         <v>1</v>
       </c>
       <c r="C41" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="D41" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E41">
         <v>0</v>
@@ -2422,24 +2651,30 @@
         <v>1</v>
       </c>
       <c r="H41" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="I41" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="J41">
+        <v>0</v>
+      </c>
+      <c r="K41">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B42">
         <v>1</v>
       </c>
       <c r="C42" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D42" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E42">
         <v>1</v>
@@ -2451,53 +2686,65 @@
         <v>1</v>
       </c>
       <c r="H42" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="I42" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="J42">
+        <v>0</v>
+      </c>
+      <c r="K42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
+        <v>84</v>
+      </c>
+      <c r="B43">
+        <v>0</v>
+      </c>
+      <c r="C43" t="s">
+        <v>144</v>
+      </c>
+      <c r="D43" t="s">
+        <v>43</v>
+      </c>
+      <c r="E43">
+        <v>0</v>
+      </c>
+      <c r="F43" s="6">
+        <v>1</v>
+      </c>
+      <c r="G43">
+        <v>1</v>
+      </c>
+      <c r="H43" t="s">
+        <v>130</v>
+      </c>
+      <c r="I43" t="s">
+        <v>136</v>
+      </c>
+      <c r="J43">
+        <v>0</v>
+      </c>
+      <c r="K43">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
         <v>86</v>
       </c>
-      <c r="B43">
-        <v>0</v>
-      </c>
-      <c r="C43" t="s">
+      <c r="B44">
+        <v>0</v>
+      </c>
+      <c r="C44" t="s">
         <v>85</v>
       </c>
-      <c r="D43" t="s">
-        <v>44</v>
-      </c>
-      <c r="E43">
-        <v>0</v>
-      </c>
-      <c r="F43" s="6">
-        <v>1</v>
-      </c>
-      <c r="G43">
-        <v>1</v>
-      </c>
-      <c r="H43" t="s">
-        <v>133</v>
-      </c>
-      <c r="I43" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A44" t="s">
-        <v>88</v>
-      </c>
-      <c r="B44">
-        <v>0</v>
-      </c>
-      <c r="C44" t="s">
-        <v>87</v>
-      </c>
       <c r="D44" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E44">
         <v>0</v>
@@ -2509,24 +2756,30 @@
         <v>1</v>
       </c>
       <c r="H44" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="I44" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="J44">
+        <v>0</v>
+      </c>
+      <c r="K44">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B45">
         <v>0</v>
       </c>
       <c r="C45" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D45" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E45">
         <v>0</v>
@@ -2538,53 +2791,65 @@
         <v>1</v>
       </c>
       <c r="H45" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="I45" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="J45">
+        <v>0</v>
+      </c>
+      <c r="K45">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
+        <v>89</v>
+      </c>
+      <c r="B46">
+        <v>1</v>
+      </c>
+      <c r="C46" t="s">
+        <v>137</v>
+      </c>
+      <c r="D46" t="s">
+        <v>63</v>
+      </c>
+      <c r="E46">
+        <v>0</v>
+      </c>
+      <c r="F46" s="6">
+        <v>1</v>
+      </c>
+      <c r="G46">
+        <v>1</v>
+      </c>
+      <c r="H46" t="s">
+        <v>130</v>
+      </c>
+      <c r="I46" t="s">
+        <v>136</v>
+      </c>
+      <c r="J46">
+        <v>0</v>
+      </c>
+      <c r="K46">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
         <v>91</v>
       </c>
-      <c r="B46">
-        <v>1</v>
-      </c>
-      <c r="C46" t="s">
-        <v>140</v>
-      </c>
-      <c r="D46" t="s">
-        <v>64</v>
-      </c>
-      <c r="E46">
-        <v>0</v>
-      </c>
-      <c r="F46" s="6">
-        <v>1</v>
-      </c>
-      <c r="G46">
-        <v>1</v>
-      </c>
-      <c r="H46" t="s">
-        <v>133</v>
-      </c>
-      <c r="I46" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A47" t="s">
-        <v>93</v>
-      </c>
       <c r="B47">
         <v>1</v>
       </c>
       <c r="C47" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D47" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E47">
         <v>0</v>
@@ -2596,24 +2861,30 @@
         <v>1</v>
       </c>
       <c r="H47" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="I47" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="J47">
+        <v>0</v>
+      </c>
+      <c r="K47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B48">
         <v>1</v>
       </c>
       <c r="C48" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D48" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E48">
         <v>0</v>
@@ -2625,24 +2896,30 @@
         <v>1</v>
       </c>
       <c r="H48" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="I48" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="J48">
+        <v>0</v>
+      </c>
+      <c r="K48">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B49">
         <v>1</v>
       </c>
       <c r="C49" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D49" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E49">
         <v>0</v>
@@ -2654,24 +2931,30 @@
         <v>1</v>
       </c>
       <c r="H49" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="I49" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="J49">
+        <v>0</v>
+      </c>
+      <c r="K49">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B50">
         <v>1</v>
       </c>
       <c r="C50" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="D50" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E50">
         <v>0</v>
@@ -2683,24 +2966,30 @@
         <v>1</v>
       </c>
       <c r="H50" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="I50" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+      <c r="J50">
+        <v>0</v>
+      </c>
+      <c r="K50">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B51">
         <v>1</v>
       </c>
       <c r="C51" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D51" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E51">
         <v>0</v>
@@ -2712,24 +3001,30 @@
         <v>1</v>
       </c>
       <c r="H51" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="I51" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
+        <v>135</v>
+      </c>
+      <c r="J51">
+        <v>0</v>
+      </c>
+      <c r="K51">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B52">
         <v>1</v>
       </c>
       <c r="C52" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D52" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E52">
         <v>0</v>
@@ -2741,24 +3036,30 @@
         <v>1</v>
       </c>
       <c r="H52" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="I52" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.2">
+        <v>135</v>
+      </c>
+      <c r="J52">
+        <v>0</v>
+      </c>
+      <c r="K52">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B53">
         <v>-1</v>
       </c>
       <c r="C53" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D53" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E53">
         <v>0</v>
@@ -2770,24 +3071,27 @@
         <v>0</v>
       </c>
       <c r="H53" t="s">
-        <v>142</v>
-      </c>
-      <c r="J53" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.2">
+        <v>139</v>
+      </c>
+      <c r="J53">
+        <v>1</v>
+      </c>
+      <c r="K53">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B54">
         <v>1</v>
       </c>
       <c r="C54" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D54" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E54">
         <v>0</v>
@@ -2799,24 +3103,27 @@
         <v>0</v>
       </c>
       <c r="H54" t="s">
-        <v>142</v>
-      </c>
-      <c r="J54" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.2">
+        <v>139</v>
+      </c>
+      <c r="J54">
+        <v>1</v>
+      </c>
+      <c r="K54">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B55">
         <v>1</v>
       </c>
       <c r="C55" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D55" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E55">
         <v>0</v>
@@ -2828,24 +3135,27 @@
         <v>0</v>
       </c>
       <c r="H55" t="s">
-        <v>142</v>
-      </c>
-      <c r="J55" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.2">
+        <v>139</v>
+      </c>
+      <c r="J55">
+        <v>1</v>
+      </c>
+      <c r="K55">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B56">
         <v>-1</v>
       </c>
       <c r="C56" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D56" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E56">
         <v>0</v>
@@ -2857,24 +3167,27 @@
         <v>0</v>
       </c>
       <c r="H56" t="s">
-        <v>142</v>
-      </c>
-      <c r="J56" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.2">
+        <v>139</v>
+      </c>
+      <c r="J56">
+        <v>1</v>
+      </c>
+      <c r="K56">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B57">
         <v>0</v>
       </c>
       <c r="C57" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="D57" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E57">
         <v>0</v>
@@ -2886,24 +3199,27 @@
         <v>1</v>
       </c>
       <c r="H57" t="s">
-        <v>143</v>
-      </c>
-      <c r="J57" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.2">
+        <v>140</v>
+      </c>
+      <c r="J57">
+        <v>1</v>
+      </c>
+      <c r="K57">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B58">
         <v>0</v>
       </c>
       <c r="C58" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D58" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E58">
         <v>0</v>
@@ -2915,24 +3231,27 @@
         <v>1</v>
       </c>
       <c r="H58" t="s">
-        <v>143</v>
-      </c>
-      <c r="J58" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.2">
+        <v>140</v>
+      </c>
+      <c r="J58">
+        <v>1</v>
+      </c>
+      <c r="K58">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B59">
         <v>0</v>
       </c>
       <c r="C59" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D59" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E59">
         <v>0</v>
@@ -2944,24 +3263,27 @@
         <v>1</v>
       </c>
       <c r="H59" t="s">
-        <v>143</v>
-      </c>
-      <c r="J59" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.2">
+        <v>140</v>
+      </c>
+      <c r="J59">
+        <v>1</v>
+      </c>
+      <c r="K59">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B60">
         <v>0</v>
       </c>
       <c r="C60" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D60" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E60">
         <v>0</v>
@@ -2973,24 +3295,27 @@
         <v>1</v>
       </c>
       <c r="H60" t="s">
-        <v>143</v>
-      </c>
-      <c r="J60" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.2">
+        <v>140</v>
+      </c>
+      <c r="J60">
+        <v>1</v>
+      </c>
+      <c r="K60">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B61">
         <v>0</v>
       </c>
       <c r="C61" s="4" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D61" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E61">
         <v>0</v>
@@ -3002,19 +3327,22 @@
         <v>1</v>
       </c>
       <c r="H61" t="s">
-        <v>143</v>
-      </c>
-      <c r="J61" t="s">
-        <v>124</v>
+        <v>140</v>
+      </c>
+      <c r="J61">
+        <v>1</v>
+      </c>
+      <c r="K61">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L3:L8" xr:uid="{A1296866-C643-430F-9178-AD2520CDAA44}">
-      <formula1>$L$2:$L$8</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M3:M8" xr:uid="{A1296866-C643-430F-9178-AD2520CDAA44}">
+      <formula1>$M$2:$M$8</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D3:D61" xr:uid="{1643AB3D-26ED-4117-AB07-6DC5F748532F}">
-      <formula1>$L$3:$L$8</formula1>
+      <formula1>$M$3:$M$8</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>